<commit_message>
Se corrigio el problema de la acumulacion por escoltas identificada por don carlos y socializada el dia 14 de octubre, se valida la informacion de por el aux y el coord de sistemas y desarrollo
</commit_message>
<xml_diff>
--- a/public/assets/Acompañamiento.xlsx
+++ b/public/assets/Acompañamiento.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SISTEMAS\Documents\Angular\PDV\public\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{639FE4E9-10FC-41AD-8C5F-9A61430FD4F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BA2FC7A-2392-4063-90AD-130C6BABE69E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Consignaciones" sheetId="1" r:id="rId1"/>
@@ -6930,9 +6930,9 @@
     <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -75910,5 +75910,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>